<commit_message>
updates to process-trial for s17 and s18, crossover filter
</commit_message>
<xml_diff>
--- a/results/ncbc_s17/m3/pred_peaks.xlsx
+++ b/results/ncbc_s17/m3/pred_peaks.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,17 +417,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>step_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>side</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>peak_value</t>
         </is>
@@ -455,7 +443,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.9684840440750122</v>
+        <v>0.9679632186889648</v>
       </c>
     </row>
     <row r="3">
@@ -468,7 +456,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1.128673076629639</v>
+        <v>1.120322465896606</v>
       </c>
     </row>
     <row r="4">
@@ -481,7 +469,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1.257912874221802</v>
+        <v>1.246644496917725</v>
       </c>
     </row>
     <row r="5">
@@ -494,7 +482,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1.206722259521484</v>
+        <v>1.200446009635925</v>
       </c>
     </row>
     <row r="6">
@@ -507,7 +495,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1.568269014358521</v>
+        <v>1.556840062141418</v>
       </c>
     </row>
     <row r="7">
@@ -520,7 +508,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1.479483723640442</v>
+        <v>1.469143867492676</v>
       </c>
     </row>
     <row r="8">
@@ -533,7 +521,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1.365578174591064</v>
+        <v>1.358370780944824</v>
       </c>
     </row>
     <row r="9">
@@ -546,7 +534,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1.480530023574829</v>
+        <v>1.470564603805542</v>
       </c>
     </row>
     <row r="10">
@@ -559,7 +547,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1.3652024269104</v>
+        <v>1.359296321868896</v>
       </c>
     </row>
     <row r="11">
@@ -572,7 +560,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1.449576616287231</v>
+        <v>1.433937549591064</v>
       </c>
     </row>
     <row r="12">
@@ -585,7 +573,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1.449884653091431</v>
+        <v>1.444610357284546</v>
       </c>
     </row>
     <row r="13">
@@ -598,7 +586,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1.456795454025269</v>
+        <v>1.448012232780457</v>
       </c>
     </row>
     <row r="14">
@@ -611,7 +599,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1.47496223449707</v>
+        <v>1.465895533561707</v>
       </c>
     </row>
     <row r="15">
@@ -624,7 +612,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1.420126676559448</v>
+        <v>1.411110639572144</v>
       </c>
     </row>
     <row r="16">
@@ -637,7 +625,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1.488154649734497</v>
+        <v>1.478753805160522</v>
       </c>
     </row>
     <row r="17">
@@ -650,7 +638,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1.61921501159668</v>
+        <v>1.606251239776611</v>
       </c>
     </row>
     <row r="18">
@@ -663,7 +651,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1.417291402816772</v>
+        <v>1.40166175365448</v>
       </c>
     </row>
     <row r="19">
@@ -676,7 +664,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1.347718358039856</v>
+        <v>1.340142250061035</v>
       </c>
     </row>
     <row r="20">
@@ -689,7 +677,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1.08304762840271</v>
+        <v>1.077720284461975</v>
       </c>
     </row>
     <row r="21">
@@ -702,7 +690,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1.544157028198242</v>
+        <v>1.533095240592957</v>
       </c>
     </row>
     <row r="22">
@@ -715,7 +703,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1.454210758209229</v>
+        <v>1.443429708480835</v>
       </c>
     </row>
     <row r="23">
@@ -728,7 +716,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1.436483144760132</v>
+        <v>1.427902698516846</v>
       </c>
     </row>
     <row r="24">
@@ -741,7 +729,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>1.470291376113892</v>
+        <v>1.46085524559021</v>
       </c>
     </row>
     <row r="25">
@@ -754,7 +742,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1.378983020782471</v>
+        <v>1.37041449546814</v>
       </c>
     </row>
     <row r="26">
@@ -767,7 +755,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1.415412187576294</v>
+        <v>1.408084034919739</v>
       </c>
     </row>
     <row r="27">
@@ -780,7 +768,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1.416205883026123</v>
+        <v>1.401225090026855</v>
       </c>
     </row>
     <row r="28">
@@ -793,7 +781,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1.509727001190186</v>
+        <v>1.499292373657227</v>
       </c>
     </row>
     <row r="29">
@@ -806,7 +794,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1.529552936553955</v>
+        <v>1.518187880516052</v>
       </c>
     </row>
     <row r="30">
@@ -819,7 +807,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1.376189708709717</v>
+        <v>1.366731286048889</v>
       </c>
     </row>
     <row r="31">
@@ -832,7 +820,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1.414325714111328</v>
+        <v>1.405739545822144</v>
       </c>
     </row>
     <row r="32">
@@ -845,7 +833,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1.441996097564697</v>
+        <v>1.433447599411011</v>
       </c>
     </row>
     <row r="33">
@@ -858,7 +846,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1.396477699279785</v>
+        <v>1.390209913253784</v>
       </c>
     </row>
     <row r="34">
@@ -871,7 +859,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1.556638956069946</v>
+        <v>1.545272946357727</v>
       </c>
     </row>
     <row r="35">
@@ -884,7 +872,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1.443168520927429</v>
+        <v>1.434386014938354</v>
       </c>
     </row>
     <row r="36">
@@ -897,7 +885,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1.422912120819092</v>
+        <v>1.413823366165161</v>
       </c>
     </row>
     <row r="37">
@@ -910,7 +898,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1.368384838104248</v>
+        <v>1.361106276512146</v>
       </c>
     </row>
     <row r="38">
@@ -923,7 +911,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1.336604595184326</v>
+        <v>1.331238746643066</v>
       </c>
     </row>
     <row r="39">
@@ -936,7 +924,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1.33749794960022</v>
+        <v>1.332293510437012</v>
       </c>
     </row>
     <row r="40">
@@ -949,7 +937,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>1.400126099586487</v>
+        <v>1.393792867660522</v>
       </c>
     </row>
     <row r="41">
@@ -962,7 +950,7 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>1.292559027671814</v>
+        <v>1.292104959487915</v>
       </c>
     </row>
     <row r="42">
@@ -975,7 +963,7 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1.47314977645874</v>
+        <v>1.463055849075317</v>
       </c>
     </row>
     <row r="43">
@@ -988,7 +976,7 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>1.358611583709717</v>
+        <v>1.352872610092163</v>
       </c>
     </row>
     <row r="44">
@@ -1001,7 +989,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>1.387714147567749</v>
+        <v>1.38517701625824</v>
       </c>
     </row>
     <row r="45">
@@ -1014,7 +1002,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>1.473505735397339</v>
+        <v>1.464708089828491</v>
       </c>
     </row>
     <row r="46">
@@ -1027,7 +1015,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1.403038263320923</v>
+        <v>1.395347476005554</v>
       </c>
     </row>
     <row r="47">
@@ -1040,7 +1028,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1.434889674186707</v>
+        <v>1.42683732509613</v>
       </c>
     </row>
     <row r="48">
@@ -1053,7 +1041,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>1.543066024780273</v>
+        <v>1.531316518783569</v>
       </c>
     </row>
     <row r="49">
@@ -1066,7 +1054,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1.401178598403931</v>
+        <v>1.394584655761719</v>
       </c>
     </row>
     <row r="50">
@@ -1079,7 +1067,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>1.456658840179443</v>
+        <v>1.446938753128052</v>
       </c>
     </row>
     <row r="51">
@@ -1092,7 +1080,7 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>1.434158802032471</v>
+        <v>1.426117539405823</v>
       </c>
     </row>
     <row r="52">
@@ -1105,7 +1093,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>1.408339738845825</v>
+        <v>1.400954723358154</v>
       </c>
     </row>
     <row r="53">
@@ -1118,7 +1106,7 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>1.421535849571228</v>
+        <v>1.413837432861328</v>
       </c>
     </row>
     <row r="54">
@@ -1131,7 +1119,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>1.430644273757935</v>
+        <v>1.422211647033691</v>
       </c>
     </row>
     <row r="55">
@@ -1144,7 +1132,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>1.367297768592834</v>
+        <v>1.358802556991577</v>
       </c>
     </row>
     <row r="56">
@@ -1157,7 +1145,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>1.450518608093262</v>
+        <v>1.44136905670166</v>
       </c>
     </row>
     <row r="57">
@@ -1170,7 +1158,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>1.332394361495972</v>
+        <v>1.326383590698242</v>
       </c>
     </row>
     <row r="58">
@@ -1183,7 +1171,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>1.349074840545654</v>
+        <v>1.3463454246521</v>
       </c>
     </row>
     <row r="59">
@@ -1196,7 +1184,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>1.392575979232788</v>
+        <v>1.385594725608826</v>
       </c>
     </row>
     <row r="60">
@@ -1209,7 +1197,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>1.494990348815918</v>
+        <v>1.483062386512756</v>
       </c>
     </row>
     <row r="61">
@@ -1222,7 +1210,7 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>1.396053910255432</v>
+        <v>1.388984799385071</v>
       </c>
     </row>
     <row r="62">
@@ -1235,7 +1223,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>1.357510328292847</v>
+        <v>1.352493524551392</v>
       </c>
     </row>
     <row r="63">
@@ -1248,7 +1236,7 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>1.424330234527588</v>
+        <v>1.416983366012573</v>
       </c>
     </row>
     <row r="64">
@@ -1261,7 +1249,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1.434406399726868</v>
+        <v>1.426382064819336</v>
       </c>
     </row>
     <row r="65">
@@ -1274,7 +1262,7 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>1.492952585220337</v>
+        <v>1.482942342758179</v>
       </c>
     </row>
     <row r="66">
@@ -1287,7 +1275,7 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1.345944762229919</v>
+        <v>1.340526580810547</v>
       </c>
     </row>
     <row r="67">
@@ -1300,7 +1288,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>1.482059121131897</v>
+        <v>1.472812175750732</v>
       </c>
     </row>
     <row r="68">
@@ -1313,7 +1301,7 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>1.4575035572052</v>
+        <v>1.448878765106201</v>
       </c>
     </row>
     <row r="69">
@@ -1326,7 +1314,7 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>1.215949058532715</v>
+        <v>1.214131116867065</v>
       </c>
     </row>
     <row r="70">
@@ -1339,7 +1327,7 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>1.223404765129089</v>
+        <v>1.215542554855347</v>
       </c>
     </row>
     <row r="71">
@@ -1352,7 +1340,7 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>1.515132427215576</v>
+        <v>1.502673506736755</v>
       </c>
     </row>
     <row r="72">
@@ -1365,7 +1353,7 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1.391829490661621</v>
+        <v>1.384398221969604</v>
       </c>
     </row>
     <row r="73">
@@ -1378,7 +1366,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>1.365351676940918</v>
+        <v>1.355515718460083</v>
       </c>
     </row>
     <row r="74">
@@ -1391,7 +1379,7 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>1.362615942955017</v>
+        <v>1.360714197158813</v>
       </c>
     </row>
     <row r="75">
@@ -1404,7 +1392,7 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>1.476486444473267</v>
+        <v>1.46731424331665</v>
       </c>
     </row>
     <row r="76">
@@ -1417,7 +1405,7 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>1.498660087585449</v>
+        <v>1.488505601882935</v>
       </c>
     </row>
     <row r="77">
@@ -1430,7 +1418,7 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>1.416913151741028</v>
+        <v>1.408828258514404</v>
       </c>
     </row>
     <row r="78">
@@ -1443,7 +1431,7 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>1.440343141555786</v>
+        <v>1.430973291397095</v>
       </c>
     </row>
     <row r="79">
@@ -1456,7 +1444,7 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>1.475909471511841</v>
+        <v>1.465659976005554</v>
       </c>
     </row>
     <row r="80">
@@ -1469,7 +1457,7 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>1.526879549026489</v>
+        <v>1.516010403633118</v>
       </c>
     </row>
     <row r="81">
@@ -1482,7 +1470,7 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>1.367066621780396</v>
+        <v>1.359639406204224</v>
       </c>
     </row>
     <row r="82">
@@ -1495,7 +1483,7 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>1.397300958633423</v>
+        <v>1.391253471374512</v>
       </c>
     </row>
     <row r="83">
@@ -1508,7 +1496,7 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>1.523703098297119</v>
+        <v>1.511835932731628</v>
       </c>
     </row>
     <row r="84">
@@ -1521,7 +1509,7 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>1.498656749725342</v>
+        <v>1.486750602722168</v>
       </c>
     </row>
     <row r="85">
@@ -1534,7 +1522,7 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>1.364442586898804</v>
+        <v>1.35622501373291</v>
       </c>
     </row>
     <row r="86">
@@ -1547,7 +1535,7 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>1.474766731262207</v>
+        <v>1.46791660785675</v>
       </c>
     </row>
     <row r="87">
@@ -1560,7 +1548,7 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>1.531533360481262</v>
+        <v>1.520546436309814</v>
       </c>
     </row>
     <row r="88">
@@ -1573,7 +1561,7 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>1.422423124313354</v>
+        <v>1.41468620300293</v>
       </c>
     </row>
     <row r="89">
@@ -1586,7 +1574,7 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>1.427893161773682</v>
+        <v>1.418986558914185</v>
       </c>
     </row>
     <row r="90">
@@ -1599,7 +1587,7 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>1.438862681388855</v>
+        <v>1.430705189704895</v>
       </c>
     </row>
     <row r="91">
@@ -1612,7 +1600,7 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>1.43362557888031</v>
+        <v>1.424975752830505</v>
       </c>
     </row>
     <row r="92">
@@ -1625,7 +1613,7 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>1.461263060569763</v>
+        <v>1.452543139457703</v>
       </c>
     </row>
     <row r="93">
@@ -1638,7 +1626,7 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>1.456849932670593</v>
+        <v>1.451210260391235</v>
       </c>
     </row>
     <row r="94">
@@ -1651,7 +1639,7 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>1.395874619483948</v>
+        <v>1.387630939483643</v>
       </c>
     </row>
     <row r="95">
@@ -1664,7 +1652,7 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>1.371593356132507</v>
+        <v>1.365525960922241</v>
       </c>
     </row>
     <row r="96">
@@ -1677,7 +1665,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>1.428552031517029</v>
+        <v>1.42007315158844</v>
       </c>
     </row>
     <row r="97">
@@ -1690,7 +1678,7 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>1.434150695800781</v>
+        <v>1.425530195236206</v>
       </c>
     </row>
     <row r="98">
@@ -1703,7 +1691,7 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>1.455953359603882</v>
+        <v>1.446879863739014</v>
       </c>
     </row>
     <row r="99">
@@ -1716,7 +1704,7 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>1.44001030921936</v>
+        <v>1.429463624954224</v>
       </c>
     </row>
     <row r="100">
@@ -1729,7 +1717,7 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>1.498178005218506</v>
+        <v>1.487364768981934</v>
       </c>
     </row>
     <row r="101">
@@ -1742,7 +1730,7 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>1.365315198898315</v>
+        <v>1.357264041900635</v>
       </c>
     </row>
     <row r="102">
@@ -1755,7 +1743,7 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>1.452197670936584</v>
+        <v>1.443001866340637</v>
       </c>
     </row>
     <row r="103">
@@ -1768,7 +1756,7 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>1.444779396057129</v>
+        <v>1.440442085266113</v>
       </c>
     </row>
     <row r="104">
@@ -1781,7 +1769,7 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>1.477246642112732</v>
+        <v>1.467630505561829</v>
       </c>
     </row>
     <row r="105">
@@ -1794,7 +1782,7 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>1.344197273254395</v>
+        <v>1.338823080062866</v>
       </c>
     </row>
     <row r="106">
@@ -1807,7 +1795,7 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>1.513598203659058</v>
+        <v>1.503065347671509</v>
       </c>
     </row>
     <row r="107">
@@ -1820,7 +1808,7 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>1.394698619842529</v>
+        <v>1.387778282165527</v>
       </c>
     </row>
     <row r="108">
@@ -1833,7 +1821,7 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>1.407127380371094</v>
+        <v>1.398619294166565</v>
       </c>
     </row>
     <row r="109">
@@ -1846,7 +1834,7 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>1.465505838394165</v>
+        <v>1.455515742301941</v>
       </c>
     </row>
     <row r="110">
@@ -1859,7 +1847,7 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>1.499202489852905</v>
+        <v>1.489521741867065</v>
       </c>
     </row>
     <row r="111">
@@ -1872,7 +1860,7 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>1.440060496330261</v>
+        <v>1.431694269180298</v>
       </c>
     </row>
     <row r="112">
@@ -1885,7 +1873,7 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>1.442922830581665</v>
+        <v>1.434046983718872</v>
       </c>
     </row>
     <row r="113">
@@ -1898,7 +1886,7 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>1.39191722869873</v>
+        <v>1.382765531539917</v>
       </c>
     </row>
     <row r="114">
@@ -1911,7 +1899,7 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>1.485238671302795</v>
+        <v>1.473671913146973</v>
       </c>
     </row>
     <row r="115">
@@ -1924,7 +1912,7 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>1.467715978622437</v>
+        <v>1.457669854164124</v>
       </c>
     </row>
     <row r="116">
@@ -1937,7 +1925,7 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>1.406728863716125</v>
+        <v>1.398802518844604</v>
       </c>
     </row>
     <row r="117">
@@ -1950,7 +1938,7 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>1.365972280502319</v>
+        <v>1.362080335617065</v>
       </c>
     </row>
     <row r="118">
@@ -1963,7 +1951,7 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>1.467170000076294</v>
+        <v>1.458300352096558</v>
       </c>
     </row>
     <row r="119">
@@ -1976,7 +1964,7 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>1.511236548423767</v>
+        <v>1.501875162124634</v>
       </c>
     </row>
     <row r="120">
@@ -1989,7 +1977,7 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>1.408928394317627</v>
+        <v>1.400374412536621</v>
       </c>
     </row>
     <row r="121">
@@ -2002,7 +1990,7 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>1.392813682556152</v>
+        <v>1.383960127830505</v>
       </c>
     </row>
     <row r="122">
@@ -2015,7 +2003,7 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>1.471813678741455</v>
+        <v>1.461667776107788</v>
       </c>
     </row>
     <row r="123">
@@ -2028,7 +2016,7 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>1.159286975860596</v>
+        <v>1.150997400283813</v>
       </c>
     </row>
     <row r="124">
@@ -2041,7 +2029,7 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>1.108785629272461</v>
+        <v>1.104357481002808</v>
       </c>
     </row>
     <row r="125">
@@ -2054,7 +2042,7 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>1.040506362915039</v>
+        <v>1.034642934799194</v>
       </c>
     </row>
     <row r="126">
@@ -2067,7 +2055,7 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>0.991730272769928</v>
+        <v>0.9911996126174927</v>
       </c>
     </row>
     <row r="127">
@@ -2080,7 +2068,7 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>1.104759454727173</v>
+        <v>1.098468780517578</v>
       </c>
     </row>
     <row r="128">
@@ -2093,7 +2081,7 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>1.13256561756134</v>
+        <v>1.12462329864502</v>
       </c>
     </row>
     <row r="129">
@@ -2106,7 +2094,7 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>1.26344358921051</v>
+        <v>1.263184547424316</v>
       </c>
     </row>
     <row r="130">
@@ -2119,7 +2107,7 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>1.44969379901886</v>
+        <v>1.436968326568604</v>
       </c>
     </row>
     <row r="131">
@@ -2132,7 +2120,7 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>1.611940860748291</v>
+        <v>1.598250865936279</v>
       </c>
     </row>
     <row r="132">
@@ -2145,7 +2133,7 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>1.478270530700684</v>
+        <v>1.474063873291016</v>
       </c>
     </row>
     <row r="133">
@@ -2158,7 +2146,7 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>1.506628632545471</v>
+        <v>1.495096445083618</v>
       </c>
     </row>
     <row r="134">
@@ -2171,7 +2159,7 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>1.546788930892944</v>
+        <v>1.534621953964233</v>
       </c>
     </row>
     <row r="135">
@@ -2184,7 +2172,7 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>1.525478005409241</v>
+        <v>1.515439987182617</v>
       </c>
     </row>
     <row r="136">
@@ -2197,7 +2185,7 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>1.467670202255249</v>
+        <v>1.456944704055786</v>
       </c>
     </row>
     <row r="137">
@@ -2210,7 +2198,7 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>1.470402956008911</v>
+        <v>1.459136724472046</v>
       </c>
     </row>
     <row r="138">
@@ -2223,7 +2211,7 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>1.494843482971191</v>
+        <v>1.482457876205444</v>
       </c>
     </row>
     <row r="139">
@@ -2236,7 +2224,7 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>1.535895347595215</v>
+        <v>1.521937608718872</v>
       </c>
     </row>
     <row r="140">
@@ -2249,7 +2237,7 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>1.507418632507324</v>
+        <v>1.494725704193115</v>
       </c>
     </row>
     <row r="141">
@@ -2262,7 +2250,7 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>1.446985006332397</v>
+        <v>1.437168598175049</v>
       </c>
     </row>
     <row r="142">
@@ -2275,7 +2263,7 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>1.486193895339966</v>
+        <v>1.473945379257202</v>
       </c>
     </row>
     <row r="143">
@@ -2288,7 +2276,7 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>1.470396518707275</v>
+        <v>1.458641290664673</v>
       </c>
     </row>
     <row r="144">
@@ -2301,7 +2289,7 @@
         </is>
       </c>
       <c r="C144" t="n">
-        <v>1.443857192993164</v>
+        <v>1.431079626083374</v>
       </c>
     </row>
     <row r="145">
@@ -2314,7 +2302,7 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>1.518890738487244</v>
+        <v>1.505907535552979</v>
       </c>
     </row>
     <row r="146">
@@ -2327,7 +2315,7 @@
         </is>
       </c>
       <c r="C146" t="n">
-        <v>1.574854254722595</v>
+        <v>1.560818314552307</v>
       </c>
     </row>
     <row r="147">
@@ -2340,7 +2328,7 @@
         </is>
       </c>
       <c r="C147" t="n">
-        <v>1.504317998886108</v>
+        <v>1.493417859077454</v>
       </c>
     </row>
     <row r="148">
@@ -2353,7 +2341,7 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>1.431613683700562</v>
+        <v>1.418957352638245</v>
       </c>
     </row>
     <row r="149">
@@ -2366,7 +2354,7 @@
         </is>
       </c>
       <c r="C149" t="n">
-        <v>1.472893118858337</v>
+        <v>1.461004972457886</v>
       </c>
     </row>
     <row r="150">
@@ -2379,7 +2367,7 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>1.587462425231934</v>
+        <v>1.581143379211426</v>
       </c>
     </row>
     <row r="151">
@@ -2392,7 +2380,7 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>1.494542121887207</v>
+        <v>1.480901479721069</v>
       </c>
     </row>
     <row r="152">
@@ -2405,7 +2393,7 @@
         </is>
       </c>
       <c r="C152" t="n">
-        <v>1.37948751449585</v>
+        <v>1.369776487350464</v>
       </c>
     </row>
     <row r="153">
@@ -2418,7 +2406,7 @@
         </is>
       </c>
       <c r="C153" t="n">
-        <v>1.546367168426514</v>
+        <v>1.531577110290527</v>
       </c>
     </row>
     <row r="154">
@@ -2431,7 +2419,7 @@
         </is>
       </c>
       <c r="C154" t="n">
-        <v>1.502922296524048</v>
+        <v>1.489497184753418</v>
       </c>
     </row>
     <row r="155">
@@ -2444,7 +2432,7 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>1.448026657104492</v>
+        <v>1.434326648712158</v>
       </c>
     </row>
     <row r="156">
@@ -2457,7 +2445,7 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>1.540512561798096</v>
+        <v>1.527465105056763</v>
       </c>
     </row>
     <row r="157">
@@ -2470,7 +2458,7 @@
         </is>
       </c>
       <c r="C157" t="n">
-        <v>1.505802154541016</v>
+        <v>1.493674635887146</v>
       </c>
     </row>
     <row r="158">
@@ -2483,7 +2471,7 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>1.506850719451904</v>
+        <v>1.494453907012939</v>
       </c>
     </row>
     <row r="159">
@@ -2496,7 +2484,7 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>1.48221230506897</v>
+        <v>1.470439195632935</v>
       </c>
     </row>
     <row r="160">
@@ -2509,7 +2497,7 @@
         </is>
       </c>
       <c r="C160" t="n">
-        <v>1.572075963020325</v>
+        <v>1.557756900787354</v>
       </c>
     </row>
     <row r="161">
@@ -2522,7 +2510,7 @@
         </is>
       </c>
       <c r="C161" t="n">
-        <v>1.548215866088867</v>
+        <v>1.535498142242432</v>
       </c>
     </row>
     <row r="162">
@@ -2535,7 +2523,7 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>1.585817813873291</v>
+        <v>1.571303129196167</v>
       </c>
     </row>
     <row r="163">
@@ -2548,7 +2536,7 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>1.500565409660339</v>
+        <v>1.488487958908081</v>
       </c>
     </row>
     <row r="164">
@@ -2561,7 +2549,7 @@
         </is>
       </c>
       <c r="C164" t="n">
-        <v>1.532385945320129</v>
+        <v>1.519638538360596</v>
       </c>
     </row>
     <row r="165">
@@ -2574,7 +2562,7 @@
         </is>
       </c>
       <c r="C165" t="n">
-        <v>1.51384973526001</v>
+        <v>1.501011490821838</v>
       </c>
     </row>
     <row r="166">
@@ -2587,7 +2575,7 @@
         </is>
       </c>
       <c r="C166" t="n">
-        <v>1.531311511993408</v>
+        <v>1.51835036277771</v>
       </c>
     </row>
     <row r="167">
@@ -2600,7 +2588,7 @@
         </is>
       </c>
       <c r="C167" t="n">
-        <v>1.523796796798706</v>
+        <v>1.510700464248657</v>
       </c>
     </row>
     <row r="168">
@@ -2613,7 +2601,7 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>1.513733386993408</v>
+        <v>1.500787496566772</v>
       </c>
     </row>
     <row r="169">
@@ -2626,7 +2614,7 @@
         </is>
       </c>
       <c r="C169" t="n">
-        <v>1.486662864685059</v>
+        <v>1.474495410919189</v>
       </c>
     </row>
     <row r="170">
@@ -2639,7 +2627,7 @@
         </is>
       </c>
       <c r="C170" t="n">
-        <v>1.469170093536377</v>
+        <v>1.457036972045898</v>
       </c>
     </row>
     <row r="171">
@@ -2652,7 +2640,7 @@
         </is>
       </c>
       <c r="C171" t="n">
-        <v>1.521541357040405</v>
+        <v>1.509068727493286</v>
       </c>
     </row>
     <row r="172">
@@ -2665,7 +2653,7 @@
         </is>
       </c>
       <c r="C172" t="n">
-        <v>1.516641616821289</v>
+        <v>1.503715515136719</v>
       </c>
     </row>
     <row r="173">
@@ -2678,7 +2666,7 @@
         </is>
       </c>
       <c r="C173" t="n">
-        <v>1.538089513778687</v>
+        <v>1.52413022518158</v>
       </c>
     </row>
     <row r="174">
@@ -2691,7 +2679,7 @@
         </is>
       </c>
       <c r="C174" t="n">
-        <v>1.511134624481201</v>
+        <v>1.498255014419556</v>
       </c>
     </row>
     <row r="175">
@@ -2704,7 +2692,7 @@
         </is>
       </c>
       <c r="C175" t="n">
-        <v>1.532499551773071</v>
+        <v>1.520419836044312</v>
       </c>
     </row>
     <row r="176">
@@ -2717,7 +2705,7 @@
         </is>
       </c>
       <c r="C176" t="n">
-        <v>1.545687437057495</v>
+        <v>1.531345367431641</v>
       </c>
     </row>
     <row r="177">
@@ -2730,7 +2718,7 @@
         </is>
       </c>
       <c r="C177" t="n">
-        <v>1.505273461341858</v>
+        <v>1.492971420288086</v>
       </c>
     </row>
     <row r="178">
@@ -2743,7 +2731,7 @@
         </is>
       </c>
       <c r="C178" t="n">
-        <v>1.524534702301025</v>
+        <v>1.511764287948608</v>
       </c>
     </row>
     <row r="179">
@@ -2756,7 +2744,7 @@
         </is>
       </c>
       <c r="C179" t="n">
-        <v>1.504773378372192</v>
+        <v>1.492147445678711</v>
       </c>
     </row>
     <row r="180">
@@ -2769,7 +2757,7 @@
         </is>
       </c>
       <c r="C180" t="n">
-        <v>1.503730773925781</v>
+        <v>1.491462469100952</v>
       </c>
     </row>
     <row r="181">
@@ -2782,7 +2770,7 @@
         </is>
       </c>
       <c r="C181" t="n">
-        <v>1.450990319252014</v>
+        <v>1.444363951683044</v>
       </c>
     </row>
     <row r="182">
@@ -2795,7 +2783,7 @@
         </is>
       </c>
       <c r="C182" t="n">
-        <v>1.531259655952454</v>
+        <v>1.520291328430176</v>
       </c>
     </row>
     <row r="183">
@@ -2808,7 +2796,7 @@
         </is>
       </c>
       <c r="C183" t="n">
-        <v>1.490679979324341</v>
+        <v>1.477847814559937</v>
       </c>
     </row>
     <row r="184">
@@ -2821,7 +2809,7 @@
         </is>
       </c>
       <c r="C184" t="n">
-        <v>1.554606437683105</v>
+        <v>1.541297078132629</v>
       </c>
     </row>
     <row r="185">
@@ -2834,7 +2822,7 @@
         </is>
       </c>
       <c r="C185" t="n">
-        <v>1.551596641540527</v>
+        <v>1.539482593536377</v>
       </c>
     </row>
     <row r="186">
@@ -2847,7 +2835,7 @@
         </is>
       </c>
       <c r="C186" t="n">
-        <v>1.444492936134338</v>
+        <v>1.435956358909607</v>
       </c>
     </row>
     <row r="187">
@@ -2860,7 +2848,7 @@
         </is>
       </c>
       <c r="C187" t="n">
-        <v>1.454714059829712</v>
+        <v>1.445568799972534</v>
       </c>
     </row>
     <row r="188">
@@ -2873,7 +2861,7 @@
         </is>
       </c>
       <c r="C188" t="n">
-        <v>1.525697946548462</v>
+        <v>1.513243198394775</v>
       </c>
     </row>
     <row r="189">
@@ -2886,7 +2874,7 @@
         </is>
       </c>
       <c r="C189" t="n">
-        <v>1.525177717208862</v>
+        <v>1.5126131772995</v>
       </c>
     </row>
     <row r="190">
@@ -2899,7 +2887,7 @@
         </is>
       </c>
       <c r="C190" t="n">
-        <v>1.560603618621826</v>
+        <v>1.547142267227173</v>
       </c>
     </row>
     <row r="191">
@@ -2912,7 +2900,7 @@
         </is>
       </c>
       <c r="C191" t="n">
-        <v>1.512676239013672</v>
+        <v>1.500279784202576</v>
       </c>
     </row>
     <row r="192">
@@ -2925,7 +2913,7 @@
         </is>
       </c>
       <c r="C192" t="n">
-        <v>1.557597875595093</v>
+        <v>1.543634653091431</v>
       </c>
     </row>
     <row r="193">
@@ -2938,7 +2926,7 @@
         </is>
       </c>
       <c r="C193" t="n">
-        <v>1.487017035484314</v>
+        <v>1.475122213363647</v>
       </c>
     </row>
     <row r="194">
@@ -2951,7 +2939,7 @@
         </is>
       </c>
       <c r="C194" t="n">
-        <v>1.307046890258789</v>
+        <v>1.297631978988647</v>
       </c>
     </row>
     <row r="195">
@@ -2964,7 +2952,7 @@
         </is>
       </c>
       <c r="C195" t="n">
-        <v>1.473508477210999</v>
+        <v>1.461427450180054</v>
       </c>
     </row>
     <row r="196">
@@ -2977,7 +2965,7 @@
         </is>
       </c>
       <c r="C196" t="n">
-        <v>1.539461493492126</v>
+        <v>1.52806282043457</v>
       </c>
     </row>
     <row r="197">
@@ -2990,7 +2978,7 @@
         </is>
       </c>
       <c r="C197" t="n">
-        <v>1.515776634216309</v>
+        <v>1.50344979763031</v>
       </c>
     </row>
     <row r="198">
@@ -3003,7 +2991,7 @@
         </is>
       </c>
       <c r="C198" t="n">
-        <v>1.494045495986938</v>
+        <v>1.481741666793823</v>
       </c>
     </row>
     <row r="199">
@@ -3016,7 +3004,7 @@
         </is>
       </c>
       <c r="C199" t="n">
-        <v>1.491807222366333</v>
+        <v>1.479692935943604</v>
       </c>
     </row>
     <row r="200">
@@ -3029,7 +3017,7 @@
         </is>
       </c>
       <c r="C200" t="n">
-        <v>1.525342345237732</v>
+        <v>1.512507915496826</v>
       </c>
     </row>
     <row r="201">
@@ -3042,7 +3030,7 @@
         </is>
       </c>
       <c r="C201" t="n">
-        <v>1.529377341270447</v>
+        <v>1.516937017440796</v>
       </c>
     </row>
     <row r="202">
@@ -3055,7 +3043,7 @@
         </is>
       </c>
       <c r="C202" t="n">
-        <v>1.494364023208618</v>
+        <v>1.482523202896118</v>
       </c>
     </row>
     <row r="203">
@@ -3068,7 +3056,7 @@
         </is>
       </c>
       <c r="C203" t="n">
-        <v>1.544695854187012</v>
+        <v>1.531636834144592</v>
       </c>
     </row>
     <row r="204">
@@ -3081,7 +3069,7 @@
         </is>
       </c>
       <c r="C204" t="n">
-        <v>1.53571605682373</v>
+        <v>1.522735834121704</v>
       </c>
     </row>
     <row r="205">
@@ -3094,7 +3082,7 @@
         </is>
       </c>
       <c r="C205" t="n">
-        <v>1.533390283584595</v>
+        <v>1.521740198135376</v>
       </c>
     </row>
     <row r="206">
@@ -3107,7 +3095,7 @@
         </is>
       </c>
       <c r="C206" t="n">
-        <v>1.484526038169861</v>
+        <v>1.472743630409241</v>
       </c>
     </row>
     <row r="207">
@@ -3120,7 +3108,7 @@
         </is>
       </c>
       <c r="C207" t="n">
-        <v>1.500606775283813</v>
+        <v>1.488217353820801</v>
       </c>
     </row>
     <row r="208">
@@ -3133,7 +3121,7 @@
         </is>
       </c>
       <c r="C208" t="n">
-        <v>1.562206029891968</v>
+        <v>1.549822807312012</v>
       </c>
     </row>
     <row r="209">
@@ -3146,7 +3134,7 @@
         </is>
       </c>
       <c r="C209" t="n">
-        <v>1.540609121322632</v>
+        <v>1.527408599853516</v>
       </c>
     </row>
     <row r="210">
@@ -3159,7 +3147,7 @@
         </is>
       </c>
       <c r="C210" t="n">
-        <v>1.535618782043457</v>
+        <v>1.522212266921997</v>
       </c>
     </row>
     <row r="211">
@@ -3172,7 +3160,7 @@
         </is>
       </c>
       <c r="C211" t="n">
-        <v>1.474566578865051</v>
+        <v>1.464052081108093</v>
       </c>
     </row>
     <row r="212">
@@ -3185,7 +3173,7 @@
         </is>
       </c>
       <c r="C212" t="n">
-        <v>1.571473836898804</v>
+        <v>1.557510018348694</v>
       </c>
     </row>
     <row r="213">
@@ -3198,7 +3186,7 @@
         </is>
       </c>
       <c r="C213" t="n">
-        <v>1.504527449607849</v>
+        <v>1.492189526557922</v>
       </c>
     </row>
     <row r="214">
@@ -3211,7 +3199,7 @@
         </is>
       </c>
       <c r="C214" t="n">
-        <v>1.521105527877808</v>
+        <v>1.509731411933899</v>
       </c>
     </row>
     <row r="215">
@@ -3224,7 +3212,7 @@
         </is>
       </c>
       <c r="C215" t="n">
-        <v>1.49227499961853</v>
+        <v>1.480384588241577</v>
       </c>
     </row>
     <row r="216">
@@ -3237,7 +3225,7 @@
         </is>
       </c>
       <c r="C216" t="n">
-        <v>1.501325488090515</v>
+        <v>1.489388108253479</v>
       </c>
     </row>
     <row r="217">
@@ -3250,7 +3238,7 @@
         </is>
       </c>
       <c r="C217" t="n">
-        <v>1.486009955406189</v>
+        <v>1.472968935966492</v>
       </c>
     </row>
     <row r="218">
@@ -3263,7 +3251,7 @@
         </is>
       </c>
       <c r="C218" t="n">
-        <v>1.4753497838974</v>
+        <v>1.463375926017761</v>
       </c>
     </row>
     <row r="219">
@@ -3276,7 +3264,7 @@
         </is>
       </c>
       <c r="C219" t="n">
-        <v>1.514074087142944</v>
+        <v>1.501230955123901</v>
       </c>
     </row>
     <row r="220">
@@ -3289,7 +3277,7 @@
         </is>
       </c>
       <c r="C220" t="n">
-        <v>1.523546695709229</v>
+        <v>1.510726928710938</v>
       </c>
     </row>
     <row r="221">
@@ -3302,7 +3290,7 @@
         </is>
       </c>
       <c r="C221" t="n">
-        <v>1.463852763175964</v>
+        <v>1.454486846923828</v>
       </c>
     </row>
     <row r="222">
@@ -3315,7 +3303,7 @@
         </is>
       </c>
       <c r="C222" t="n">
-        <v>1.494296789169312</v>
+        <v>1.482502698898315</v>
       </c>
     </row>
     <row r="223">
@@ -3328,7 +3316,7 @@
         </is>
       </c>
       <c r="C223" t="n">
-        <v>1.524410486221313</v>
+        <v>1.512987852096558</v>
       </c>
     </row>
     <row r="224">
@@ -3341,7 +3329,7 @@
         </is>
       </c>
       <c r="C224" t="n">
-        <v>1.490420341491699</v>
+        <v>1.478087902069092</v>
       </c>
     </row>
     <row r="225">
@@ -3354,7 +3342,7 @@
         </is>
       </c>
       <c r="C225" t="n">
-        <v>1.486169934272766</v>
+        <v>1.474215984344482</v>
       </c>
     </row>
     <row r="226">
@@ -3367,7 +3355,7 @@
         </is>
       </c>
       <c r="C226" t="n">
-        <v>1.461710453033447</v>
+        <v>1.450123071670532</v>
       </c>
     </row>
     <row r="227">
@@ -3380,7 +3368,7 @@
         </is>
       </c>
       <c r="C227" t="n">
-        <v>1.463991641998291</v>
+        <v>1.452398300170898</v>
       </c>
     </row>
     <row r="228">
@@ -3393,7 +3381,7 @@
         </is>
       </c>
       <c r="C228" t="n">
-        <v>1.465746879577637</v>
+        <v>1.453113555908203</v>
       </c>
     </row>
     <row r="229">
@@ -3406,7 +3394,7 @@
         </is>
       </c>
       <c r="C229" t="n">
-        <v>1.563671350479126</v>
+        <v>1.54992139339447</v>
       </c>
     </row>
     <row r="230">
@@ -3419,7 +3407,7 @@
         </is>
       </c>
       <c r="C230" t="n">
-        <v>1.519134998321533</v>
+        <v>1.505604028701782</v>
       </c>
     </row>
     <row r="231">
@@ -3432,7 +3420,7 @@
         </is>
       </c>
       <c r="C231" t="n">
-        <v>1.482635259628296</v>
+        <v>1.470703601837158</v>
       </c>
     </row>
     <row r="232">
@@ -3445,7 +3433,7 @@
         </is>
       </c>
       <c r="C232" t="n">
-        <v>1.506714105606079</v>
+        <v>1.494616746902466</v>
       </c>
     </row>
     <row r="233">
@@ -3458,7 +3446,7 @@
         </is>
       </c>
       <c r="C233" t="n">
-        <v>1.533901929855347</v>
+        <v>1.520991086959839</v>
       </c>
     </row>
     <row r="234">
@@ -3471,7 +3459,7 @@
         </is>
       </c>
       <c r="C234" t="n">
-        <v>1.527758836746216</v>
+        <v>1.514833450317383</v>
       </c>
     </row>
     <row r="235">
@@ -3484,7 +3472,7 @@
         </is>
       </c>
       <c r="C235" t="n">
-        <v>1.479214429855347</v>
+        <v>1.467517375946045</v>
       </c>
     </row>
     <row r="236">
@@ -3497,7 +3485,7 @@
         </is>
       </c>
       <c r="C236" t="n">
-        <v>1.492748737335205</v>
+        <v>1.481241464614868</v>
       </c>
     </row>
     <row r="237">
@@ -3510,7 +3498,7 @@
         </is>
       </c>
       <c r="C237" t="n">
-        <v>1.474885225296021</v>
+        <v>1.465239286422729</v>
       </c>
     </row>
     <row r="238">
@@ -3523,7 +3511,7 @@
         </is>
       </c>
       <c r="C238" t="n">
-        <v>1.562540292739868</v>
+        <v>1.548254728317261</v>
       </c>
     </row>
     <row r="239">
@@ -3536,7 +3524,7 @@
         </is>
       </c>
       <c r="C239" t="n">
-        <v>1.552550435066223</v>
+        <v>1.539844751358032</v>
       </c>
     </row>
     <row r="240">
@@ -3549,7 +3537,7 @@
         </is>
       </c>
       <c r="C240" t="n">
-        <v>1.529362916946411</v>
+        <v>1.516114354133606</v>
       </c>
     </row>
     <row r="241">
@@ -3562,7 +3550,7 @@
         </is>
       </c>
       <c r="C241" t="n">
-        <v>1.451372146606445</v>
+        <v>1.440023422241211</v>
       </c>
     </row>
     <row r="242">
@@ -3575,7 +3563,7 @@
         </is>
       </c>
       <c r="C242" t="n">
-        <v>1.535079956054688</v>
+        <v>1.522639513015747</v>
       </c>
     </row>
     <row r="243">
@@ -3588,7 +3576,7 @@
         </is>
       </c>
       <c r="C243" t="n">
-        <v>1.466826677322388</v>
+        <v>1.45509147644043</v>
       </c>
     </row>
     <row r="244">
@@ -3601,7 +3589,7 @@
         </is>
       </c>
       <c r="C244" t="n">
-        <v>1.547827482223511</v>
+        <v>1.534887075424194</v>
       </c>
     </row>
     <row r="245">
@@ -3614,7 +3602,7 @@
         </is>
       </c>
       <c r="C245" t="n">
-        <v>1.496526718139648</v>
+        <v>1.48633337020874</v>
       </c>
     </row>
     <row r="246">
@@ -3627,7 +3615,7 @@
         </is>
       </c>
       <c r="C246" t="n">
-        <v>1.527923345565796</v>
+        <v>1.515576124191284</v>
       </c>
     </row>
     <row r="247">
@@ -3640,7 +3628,7 @@
         </is>
       </c>
       <c r="C247" t="n">
-        <v>1.282016277313232</v>
+        <v>1.281120538711548</v>
       </c>
     </row>
     <row r="248">
@@ -3653,7 +3641,7 @@
         </is>
       </c>
       <c r="C248" t="n">
-        <v>1.166629791259766</v>
+        <v>1.157040357589722</v>
       </c>
     </row>
     <row r="249">
@@ -3666,7 +3654,7 @@
         </is>
       </c>
       <c r="C249" t="n">
-        <v>1.109516859054565</v>
+        <v>1.103151082992554</v>
       </c>
     </row>
     <row r="250">
@@ -3679,7 +3667,7 @@
         </is>
       </c>
       <c r="C250" t="n">
-        <v>1.062368750572205</v>
+        <v>1.054716110229492</v>
       </c>
     </row>
   </sheetData>

</xml_diff>